<commit_message>
DB connection fail test (?)
</commit_message>
<xml_diff>
--- a/description/TC 설계서.xlsx
+++ b/description/TC 설계서.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suresoft\Documents\sure_rust_project\description\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5763C3AF-16BC-4C5E-BE5A-0D627C7D5739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C431D473-B1BA-435E-A5F0-5BF928A3B834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44955" yWindow="4080" windowWidth="20055" windowHeight="13620" tabRatio="291" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38910" yWindow="5115" windowWidth="20205" windowHeight="14250" tabRatio="311" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="최소 TC 조합" sheetId="4" r:id="rId1"/>
@@ -7691,7 +7691,6 @@
     <mergeCell ref="G11:G14"/>
     <mergeCell ref="F15:F18"/>
     <mergeCell ref="I27:I30"/>
-    <mergeCell ref="F23:F26"/>
     <mergeCell ref="G23:G26"/>
     <mergeCell ref="C47:C50"/>
     <mergeCell ref="D47:D50"/>
@@ -7734,6 +7733,7 @@
     <mergeCell ref="F27:F30"/>
     <mergeCell ref="C23:C26"/>
     <mergeCell ref="D23:D26"/>
+    <mergeCell ref="F23:F26"/>
     <mergeCell ref="I67:I70"/>
     <mergeCell ref="J67:J70"/>
     <mergeCell ref="C63:C66"/>

</xml_diff>